<commit_message>
feat: add GUI checklist, bug reports, and evidence
</commit_message>
<xml_diff>
--- a/submissions/gui-testing/gui-checklist-profile-page.xlsx
+++ b/submissions/gui-testing/gui-checklist-profile-page.xlsx
@@ -2,10 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phạm vi" sheetId="1" r:id="R62be479204854f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tóm tắt" sheetId="2" r:id="Rfc76f32dbcfc4e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist GUI" sheetId="3" r:id="Rde5bc15aa79144a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phản biện thủ công" sheetId="4" r:id="R58c5dfefeb7e44e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tóm tắt" sheetId="2" r:id="Re4d55a58853e490a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist GUI" sheetId="3" r:id="R8fa84f8246f64606"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -45,8 +43,13 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -83,8 +86,23 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F9FC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -157,11 +175,25 @@
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -306,6 +338,42 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -358,6 +426,632 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="a758bdbb-9d7c-40af-9f25-fdf7a930f31e"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbb1d6c85bbe34a89"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1485900" cy="4857750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="34e57ce6-0fd7-47d5-b766-a1536c1dbd93"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8ec8433706694929"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="dfbb6bc4-cd58-484c-87a8-728c89840b35"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R21cb85a48f9e4c29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="ad5f7f66-13ac-48b3-9f50-77d81e764afc"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdc8894a919e74b98"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="5e096f84-d366-4b29-b66e-60f49f3fb7ad"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R503539d53da3422a"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="2076450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="767996df-017e-44a5-aac1-29d37b5d79b2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf5fd505cc2164a25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="2143125"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="ce1df0f6-4ab3-4eed-8458-f63dbd383b57"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R50ad93a47d774eed"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="1b0f3591-23fb-49ad-b55b-9bb7be27a0c2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R31473fba752749a6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="82a260b5-a3ea-4a97-b6d3-8922fa97b565"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb39afaedb3504f09"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="63b79fa6-28f9-4054-b8d9-50a2624aab6a"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf5bd2a5711634d12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="d6bcc6a3-ec94-42d9-8034-d1d6aabf7bd1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1ae93e8a4a544b7a"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="45babe1d-bc24-4578-a266-e3b62a4f7e60"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7fb302dd6cf24581"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="c2227f84-eac9-46c2-831b-8dbdf99f09eb"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c90c22dd31144d9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="5059e6e4-684f-43a2-a06a-3b6572a6752b"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R54b20732f7ac418d"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="4171950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="add66dd1-7c01-403a-8bca-c59f0fd15e49"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc7823391a2c74d10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="8174d376-e082-478c-a7fc-265059dd6eb0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R709abaceb58c4227"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1933575"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="b2cea16d-ea37-4ccd-921f-b11447f4aea8"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R317744378d2d4ccf"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="e54a8428-2799-42bd-b48a-857079911b77"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc8c6a55b64c64fcd"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="5b385c8e-bdb7-4066-81ff-393e40c7cd85"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2a151b5f2ab845fb"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="2143125"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="11cb8501-9243-4384-8e04-d0bc4938d81b"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0ea2daef0f9c447e"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="2143125"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="9a7647cb-660d-4e63-a450-ca79c990217c"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5e1c7edb02154cad"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="2143125"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="d40bdba7-f770-474b-90cb-5d703c6001bb"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbc93343b28074afe"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3429000" cy="1943100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="4f7bef17-0366-4a38-beac-155e13ef68ba"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3f3d8d1b73304813"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -573,118 +1267,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="105" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>PHẠM VI CHECKLIST GUI</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="3"/>
-      <x:c r="B2" s="3"/>
-      <x:c r="C2" s="3"/>
-      <x:c r="D2" s="3"/>
-      <x:c r="E2" s="3"/>
-      <x:c r="F2" s="3"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="17" t="str">
-        <x:v>Thuộc tính</x:v>
-      </x:c>
-      <x:c r="B4" s="17" t="str">
-        <x:v>Nội dung</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="18" t="str">
-        <x:v>Màn hình chính (tạm chọn)</x:v>
-      </x:c>
-      <x:c r="B5" s="19" t="str">
-        <x:v>Profile page</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="18" t="str">
-        <x:v>Màn hình hỗ trợ</x:v>
-      </x:c>
-      <x:c r="B6" s="19" t="str">
-        <x:v>Update profile form; Order history screen; Admin order management</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="18" t="str">
-        <x:v>Nền tảng</x:v>
-      </x:c>
-      <x:c r="B7" s="19" t="str">
-        <x:v>Web người dùng và Web Admin</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A8" s="18" t="str">
-        <x:v>Bằng chứng đã xem</x:v>
-      </x:c>
-      <x:c r="B8" s="19" t="str">
-        <x:v>README.md (SRS FR-04, FR-10, FR-11, FR-12, FR-18, FR-21–FR-24, SEC-02/03/04/06); api_specification.md; frontend-web/src/pages/Profile.jsx; frontend-web/src/App.jsx; frontend-web/src/context/AuthContext.jsx; frontend-admin/src/App.jsx; backend/server.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="18" t="str">
-        <x:v>Giả định</x:v>
-      </x:c>
-      <x:c r="B9" s="19" t="str">
-        <x:v>Người dùng chưa chỉ định màn hình chính nên Profile page được chọn tạm thời theo thứ tự danh sách.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="18" t="str">
-        <x:v>Ranh giới thực thi</x:v>
-      </x:c>
-      <x:c r="B10" s="19" t="str">
-        <x:v>Đây là checklist thiết kế; chưa chạy trên SUT và không kết luận Passed/Failed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A11" s="18" t="str">
-        <x:v>Điểm mơ hồ</x:v>
-      </x:c>
-      <x:c r="B11" s="19" t="str">
-        <x:v>Update profile form và Order history screen hiện cùng xuất hiện trong Profile.jsx nhưng được tách thành phạm vi kiểm tra theo yêu cầu người dùng.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="18" t="str">
-        <x:v>Rủi ro độ bao phủ</x:v>
-      </x:c>
-      <x:c r="B12" s="19" t="str">
-        <x:v>Một số trạng thái loading/retry/focus động chưa được đặc tả; các kỳ vọng tương ứng được ghi rõ là Heuristic.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:F2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="43" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -753,7 +1341,7 @@
       </x:c>
       <x:c r="B6" s="47" t="n">
         <x:f>COUNTIF('Checklist GUI'!$G$2:$G$53,"Passed")+COUNTIF('Checklist GUI'!$G$2:$G$53,"Failed")</x:f>
-        <x:v>0</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C6" s="45"/>
       <x:c r="D6" s="46" t="str">
@@ -771,7 +1359,7 @@
       </x:c>
       <x:c r="B7" s="47" t="n">
         <x:f>COUNTIF('Checklist GUI'!$G$2:$G$53,"Passed")</x:f>
-        <x:v>0</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C7" s="45"/>
       <x:c r="D7" s="46" t="str">
@@ -789,7 +1377,7 @@
       </x:c>
       <x:c r="B8" s="47" t="n">
         <x:f>COUNTIF('Checklist GUI'!$G$2:$G$53,"Failed")</x:f>
-        <x:v>0</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C8" s="45"/>
       <x:c r="D8" s="46" t="str">
@@ -807,20 +1395,24 @@
       </x:c>
       <x:c r="B9" s="47" t="n">
         <x:f>COUNTIF('Checklist GUI'!$G$2:$G$53,"Chưa thực hiện")</x:f>
-        <x:v>52</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="45"/>
       <x:c r="D9" s="45"/>
       <x:c r="E9" s="45"/>
       <x:c r="F9" s="45"/>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="45"/>
-      <x:c r="B10" s="45"/>
-      <x:c r="C10" s="45"/>
-      <x:c r="D10" s="45"/>
-      <x:c r="E10" s="45"/>
-      <x:c r="F10" s="45"/>
+    <x:row r="10" ht="24" hidden="0" customHeight="1">
+      <x:c r="A10" s="61" t="str">
+        <x:v>MÀN HÌNH KIỂM THỬ</x:v>
+      </x:c>
+      <x:c r="B10" s="60"/>
+      <x:c r="C10" s="60"/>
+      <x:c r="D10" s="61" t="str">
+        <x:v>CỔNG CHẤT LƯỢNG</x:v>
+      </x:c>
+      <x:c r="E10" s="60"/>
+      <x:c r="F10" s="60"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="45"/>
@@ -837,7 +1429,9 @@
       <x:c r="B12" s="17" t="str">
         <x:v>Số mục</x:v>
       </x:c>
-      <x:c r="C12" s="45"/>
+      <x:c r="C12" s="65" t="str">
+        <x:v>Vai trò phạm vi</x:v>
+      </x:c>
       <x:c r="D12" s="17" t="str">
         <x:v>Cổng chất lượng</x:v>
       </x:c>
@@ -856,7 +1450,9 @@
         <x:f>COUNTIF('Checklist GUI'!$C$2:$C$53,"Profile page")</x:f>
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C13" s="45"/>
+      <x:c r="C13" s="69" t="str">
+        <x:v>Màn hình chính</x:v>
+      </x:c>
       <x:c r="D13" s="46" t="str">
         <x:v>Tổng &gt; 40</x:v>
       </x:c>
@@ -876,7 +1472,9 @@
         <x:f>COUNTIF('Checklist GUI'!$C$2:$C$53,"Update profile form")</x:f>
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C14" s="45"/>
+      <x:c r="C14" s="69" t="str">
+        <x:v>Màn hình hỗ trợ</x:v>
+      </x:c>
       <x:c r="D14" s="46" t="str">
         <x:v>Đủ 4 IA</x:v>
       </x:c>
@@ -896,7 +1494,9 @@
         <x:f>COUNTIF('Checklist GUI'!$C$2:$C$53,"Order history screen")</x:f>
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C15" s="45"/>
+      <x:c r="C15" s="69" t="str">
+        <x:v>Màn hình hỗ trợ</x:v>
+      </x:c>
       <x:c r="D15" s="46" t="str">
         <x:v>IA-01 ≥ 10</x:v>
       </x:c>
@@ -916,7 +1516,9 @@
         <x:f>COUNTIF('Checklist GUI'!$C$2:$C$53,"Admin order management")</x:f>
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C16" s="45"/>
+      <x:c r="C16" s="69" t="str">
+        <x:v>Màn hình hỗ trợ</x:v>
+      </x:c>
       <x:c r="D16" s="46" t="str">
         <x:v>IA-02 ≥ 8</x:v>
       </x:c>
@@ -936,7 +1538,9 @@
         <x:f>COUNTIF('Checklist GUI'!$C$2:$C$53,"Nhiều màn hình")</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C17" s="45"/>
+      <x:c r="C17" s="69" t="str">
+        <x:v>Nhiều màn hình</x:v>
+      </x:c>
       <x:c r="D17" s="46" t="str">
         <x:v>IA-03 ≥ 8</x:v>
       </x:c>
@@ -963,10 +1567,14 @@
         <x:v>Tối thiểu cứng: 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="45"/>
-      <x:c r="B19" s="45"/>
-      <x:c r="C19" s="45"/>
+    <x:row r="19" ht="28" hidden="0" customHeight="1">
+      <x:c r="A19" s="70" t="str">
+        <x:v>Nền tảng</x:v>
+      </x:c>
+      <x:c r="B19" s="68" t="str">
+        <x:v>Web người dùng và Web Admin</x:v>
+      </x:c>
+      <x:c r="C19" s="68"/>
       <x:c r="D19" s="46" t="str">
         <x:v>Màn hình chính sâu nhất</x:v>
       </x:c>
@@ -978,24 +1586,32 @@
         <x:v>Profile page &gt; từng màn hình hỗ trợ</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="45"/>
-      <x:c r="B20" s="45"/>
-      <x:c r="C20" s="45"/>
+    <x:row r="20" ht="28" hidden="0" customHeight="1">
+      <x:c r="A20" s="70" t="str">
+        <x:v>Khung thời gian thực thi</x:v>
+      </x:c>
+      <x:c r="B20" s="68" t="str">
+        <x:v>28/07/2026 – 30/07/2026</x:v>
+      </x:c>
+      <x:c r="C20" s="68"/>
       <x:c r="D20" s="46" t="str">
-        <x:v>Trạng thái thiết kế hợp lệ</x:v>
+        <x:v>Trạng thái thực thi hợp lệ</x:v>
       </x:c>
       <x:c r="E20" s="49" t="str">
-        <x:f>IF(COUNTIF('Checklist GUI'!$G$2:$G$53,"Chưa thực hiện")=B5,"Đạt","Không đạt")</x:f>
         <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F20" s="50" t="str">
-        <x:v>Thiết kế chưa được gán Passed/Failed</x:v>
+        <x:f>B7&amp;" Passed, "&amp;B8&amp;" Failed, "&amp;B9&amp;" Chưa thực hiện; toàn bộ 52 mục đã được thực thi"</x:f>
+        <x:v>26 Passed, 26 Failed, 0 Chưa thực hiện; toàn bộ 52 mục đã được thực thi</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F2"/>
+    <x:mergeCell ref="A10:C10"/>
+    <x:mergeCell ref="D10:F10"/>
+    <x:mergeCell ref="B19:C19"/>
+    <x:mergeCell ref="B20:C20"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E13:E20">
     <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Đạt"/>
@@ -1005,7 +1621,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1016,8 +1632,8 @@
     <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="51.11000061035156" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1049,7 +1665,7 @@
         <x:v>Bằng chứng</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="48" hidden="0" customHeight="1">
+    <x:row r="2" ht="165" hidden="0" customHeight="1">
       <x:c r="A2" s="56" t="str">
         <x:v>GUI-001</x:v>
       </x:c>
@@ -1069,16 +1685,14 @@
         <x:v>Trang có đúng một thẻ h1 mô tả nội dung Profile page; các tiêu đề “Hồ sơ của bạn” và “Lịch sử đơn hàng” dùng cấp heading phù hợp bên dưới. FR-21.</x:v>
       </x:c>
       <x:c r="G2" s="58" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H2" s="56" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I2" s="56" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-001 — Không có h1; hai tiêu đề khu vực đều là h2.</x:v>
+      </x:c>
+      <x:c r="I2" s="56" t="str"/>
+    </x:row>
+    <x:row r="3" ht="51" hidden="0" customHeight="1">
       <x:c r="A3" s="27" t="str">
         <x:v>GUI-002</x:v>
       </x:c>
@@ -1098,16 +1712,16 @@
         <x:v>Heuristic: Hai khu vực được phân cấp rõ, căn chỉnh nhất quán, không chồng lấn và không tạo khoảng trắng bất thường.</x:v>
       </x:c>
       <x:c r="G3" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H3" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Bố cục desktop hai cột rõ ràng, không chồng lấn ở viewport mặc định.</x:v>
       </x:c>
       <x:c r="I3" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="48" hidden="0" customHeight="1">
+    <x:row r="4" ht="394.5" hidden="0" customHeight="1">
       <x:c r="A4" s="27" t="str">
         <x:v>GUI-003</x:v>
       </x:c>
@@ -1127,16 +1741,14 @@
         <x:v>Heuristic: Nội dung chuyển thành một cột, không có thành phần bị che; người dùng đọc và thao tác được mà không phải cuộn ngang toàn trang.</x:v>
       </x:c>
       <x:c r="G4" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H4" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I4" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-002 — Hai khu vực đã reflow thành một cột, nhưng viewport 390px vẫn có document scrollWidth 404px; nội dung/control bị nén và trang cuộn ngang.</x:v>
+      </x:c>
+      <x:c r="I4" s="27" t="str"/>
+    </x:row>
+    <x:row r="5" ht="78" hidden="0" customHeight="1">
       <x:c r="A5" s="27" t="str">
         <x:v>GUI-004</x:v>
       </x:c>
@@ -1156,16 +1768,16 @@
         <x:v>Heuristic: Nhãn, giá trị và nút vẫn hiển thị đầy đủ; văn bản reflow và không bị cắt hoặc đè lên nhau.</x:v>
       </x:c>
       <x:c r="G5" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H5" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Kiểm thử thủ công ở mức zoom 200%: nội dung vẫn hiển thị đầy đủ; bố cục tự reflow từ hai cột thành một cột, không ghi nhận cắt hoặc chồng lấn.</x:v>
       </x:c>
       <x:c r="I5" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="48" hidden="0" customHeight="1">
+    <x:row r="6" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A6" s="27" t="str">
         <x:v>GUI-005</x:v>
       </x:c>
@@ -1185,16 +1797,14 @@
         <x:v>Tên người dùng được hiển thị như văn bản thuần, không render HTML và không thực thi script. SEC-04.</x:v>
       </x:c>
       <x:c r="G6" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H6" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I6" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-003 — Tên chứa thẻ b được render thành phần tử HTML trong navbar.</x:v>
+      </x:c>
+      <x:c r="I6" s="27" t="str"/>
+    </x:row>
+    <x:row r="7" ht="51" hidden="0" customHeight="1">
       <x:c r="A7" s="27" t="str">
         <x:v>GUI-006</x:v>
       </x:c>
@@ -1214,16 +1824,16 @@
         <x:v>Họ Tên, Số điện thoại và Địa chỉ giao hàng mặc định của chính người dùng được điền vào đúng trường. FR-04.</x:v>
       </x:c>
       <x:c r="G7" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H7" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Họ Tên, Số điện thoại và Địa chỉ của đúng user được nạp vào form.</x:v>
       </x:c>
       <x:c r="I7" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="48" hidden="0" customHeight="1">
+    <x:row r="8" ht="37.5" hidden="0" customHeight="1">
       <x:c r="A8" s="27" t="str">
         <x:v>GUI-007</x:v>
       </x:c>
@@ -1243,16 +1853,16 @@
         <x:v>Email hiển thị để tham chiếu nhưng không thể chỉnh sửa qua giao diện. FR-04.</x:v>
       </x:c>
       <x:c r="G8" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H8" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Email hiển thị đúng và input ở trạng thái disabled.</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="48" hidden="0" customHeight="1">
+    <x:row r="9" ht="37.5" hidden="0" customHeight="1">
       <x:c r="A9" s="27" t="str">
         <x:v>GUI-008</x:v>
       </x:c>
@@ -1272,16 +1882,16 @@
         <x:v>Không có trường hoặc điều khiển cho phép người dùng tự thay đổi role. FR-04, SEC-06.</x:v>
       </x:c>
       <x:c r="G9" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H9" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Không có control role trong form Profile.</x:v>
       </x:c>
       <x:c r="I9" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="48" hidden="0" customHeight="1">
+    <x:row r="10" ht="165" hidden="0" customHeight="1">
       <x:c r="A10" s="27" t="str">
         <x:v>GUI-009</x:v>
       </x:c>
@@ -1301,16 +1911,14 @@
         <x:v>Heuristic: Mỗi nhãn được liên kết chương trình với đúng input/textarea; tên truy cập của control phản ánh nhãn hiển thị.</x:v>
       </x:c>
       <x:c r="G10" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H10" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I10" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-004 — Các input/textarea đều có labels.length=0 và không có accessible name từ nhãn.</x:v>
+      </x:c>
+      <x:c r="I10" s="27" t="str"/>
+    </x:row>
+    <x:row r="11" ht="51" hidden="0" customHeight="1">
       <x:c r="A11" s="27" t="str">
         <x:v>GUI-010</x:v>
       </x:c>
@@ -1330,16 +1938,16 @@
         <x:v>Profile page mở đúng nội dung và mục/profile link đang chọn có trạng thái active dễ nhận biết. FR-23.</x:v>
       </x:c>
       <x:c r="G11" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H11" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Đi từ navbar mở đúng /profile; link hồ sơ có kiểu highlight màu vàng.</x:v>
       </x:c>
       <x:c r="I11" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="48" hidden="0" customHeight="1">
+    <x:row r="12" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A12" s="27" t="str">
         <x:v>GUI-011</x:v>
       </x:c>
@@ -1359,16 +1967,14 @@
         <x:v>Người dùng không được xem dữ liệu hồ sơ; hệ thống đưa ra luồng xác thực rõ ràng mà không làm lộ dữ liệu cá nhân. FR-04, SEC-02.</x:v>
       </x:c>
       <x:c r="G12" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H12" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I12" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-005 — Không lộ dữ liệu nhưng nội dung chỉ có “Vui lòng đăng nhập”, không có link đăng nhập.</x:v>
+      </x:c>
+      <x:c r="I12" s="27" t="str"/>
+    </x:row>
+    <x:row r="13" ht="37.5" hidden="0" customHeight="1">
       <x:c r="A13" s="27" t="str">
         <x:v>GUI-012</x:v>
       </x:c>
@@ -1388,16 +1994,16 @@
         <x:v>Heuristic: Route vẫn hợp lệ; sau khi khôi phục phiên, nội dung hồ sơ của đúng người dùng được hiển thị hoặc có phản hồi hết phiên rõ ràng.</x:v>
       </x:c>
       <x:c r="G13" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H13" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Refresh giữ route /profile và tải lại đúng dữ liệu user.</x:v>
       </x:c>
       <x:c r="I13" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="48" hidden="0" customHeight="1">
+    <x:row r="14" ht="64.5" hidden="0" customHeight="1">
       <x:c r="A14" s="27" t="str">
         <x:v>GUI-013</x:v>
       </x:c>
@@ -1417,16 +2023,16 @@
         <x:v>Focus đi theo thứ tự từ trên xuống dưới, trái sang phải và luôn có chỉ báo focus nhìn thấy. FR-21.</x:v>
       </x:c>
       <x:c r="G14" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H14" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Kiểm thử thủ công bằng Tab: focus di chuyển tự nhiên từ navbar đến các trường trong Profile page rồi tới nút thao tác.</x:v>
       </x:c>
       <x:c r="I14" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="48" hidden="0" customHeight="1">
+    <x:row r="15" ht="175.5" hidden="0" customHeight="1">
       <x:c r="A15" s="27" t="str">
         <x:v>GUI-014</x:v>
       </x:c>
@@ -1446,16 +2052,14 @@
         <x:v>Heuristic: Có trạng thái loading nhận biết được; dữ liệu cũ hoặc vùng trống không bị hiểu nhầm là kết quả cuối cùng.</x:v>
       </x:c>
       <x:c r="G15" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H15" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I15" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-020 — Trong lúc dữ liệu hồ sơ và đơn hàng đang tải, trang chỉ hiển thị vùng trắng và không có loading state nhận biết được.</x:v>
+      </x:c>
+      <x:c r="I15" s="27" t="str"/>
+    </x:row>
+    <x:row r="16" ht="105" hidden="0" customHeight="1">
       <x:c r="A16" s="27" t="str">
         <x:v>GUI-015</x:v>
       </x:c>
@@ -1475,16 +2079,16 @@
         <x:v>Hệ thống thông báo phiên không còn hợp lệ và không hiển thị dữ liệu cá nhân; có đường quay lại luồng đăng nhập. SEC-02.</x:v>
       </x:c>
       <x:c r="G16" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H16" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Request /api/users/me bị từ chối; hệ thống hiển thị “Vui lòng đăng nhập” và không hiển thị thông tin cá nhân. Thông báo đủ để người dùng hiểu rằng cần đăng nhập lại khi phiên không còn hợp lệ.</x:v>
       </x:c>
       <x:c r="I16" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="48" hidden="0" customHeight="1">
+    <x:row r="17" ht="180.75" hidden="0" customHeight="1">
       <x:c r="A17" s="27" t="str">
         <x:v>GUI-016</x:v>
       </x:c>
@@ -1504,16 +2108,14 @@
         <x:v>Heuristic: Có thông báo lỗi thân thiện và phân biệt với trạng thái không có đơn hàng; không chỉ ghi lỗi trong console.</x:v>
       </x:c>
       <x:c r="G17" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H17" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I17" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-019 — Khi API không phản hồi, trang coi đây là chưa đăng nhập thay vì hiển thị lỗi tải thân thiện.</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="str"/>
+    </x:row>
+    <x:row r="18" ht="51" hidden="0" customHeight="1">
       <x:c r="A18" s="56" t="str">
         <x:v>GUI-017</x:v>
       </x:c>
@@ -1533,16 +2135,16 @@
         <x:v>Các nhãn “Email (Không đổi)”, “Họ Tên”, “Số điện thoại”, “Địa chỉ giao hàng” dễ đọc, căn với đúng trường và nhất quán tiếng Việt. FR-21.</x:v>
       </x:c>
       <x:c r="G18" s="58" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H18" s="56" t="str">
-        <x:v>—</x:v>
+        <x:v>Các nhãn hiển thị đúng tiếng Việt và căn theo control tương ứng.</x:v>
       </x:c>
       <x:c r="I18" s="56" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="48" hidden="0" customHeight="1">
+    <x:row r="19" ht="64.5" hidden="0" customHeight="1">
       <x:c r="A19" s="27" t="str">
         <x:v>GUI-018</x:v>
       </x:c>
@@ -1562,16 +2164,16 @@
         <x:v>Heuristic: Dấu tiếng Việt hiển thị đúng; nội dung dài không tràn khỏi input/textarea và có thể xem lại khi chỉnh sửa.</x:v>
       </x:c>
       <x:c r="G19" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H19" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Chuỗi tiếng Việt dài giữ nguyên dấu; textarea không tràn khung và input vẫn chỉnh sửa được.</x:v>
       </x:c>
       <x:c r="I19" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="48" hidden="0" customHeight="1">
+    <x:row r="20" ht="165" hidden="0" customHeight="1">
       <x:c r="A20" s="27" t="str">
         <x:v>GUI-019</x:v>
       </x:c>
@@ -1591,16 +2193,14 @@
         <x:v>Mọi trường bắt buộc theo form đều có ký hiệu * ngay cạnh nhãn; không đánh dấu trường tùy chọn là bắt buộc. FR-22.</x:v>
       </x:c>
       <x:c r="G20" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H20" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I20" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-006 — Họ Tên có required nhưng nhãn không có dấu *.</x:v>
+      </x:c>
+      <x:c r="I20" s="27" t="str"/>
+    </x:row>
+    <x:row r="21" ht="165" hidden="0" customHeight="1">
       <x:c r="A21" s="27" t="str">
         <x:v>GUI-020</x:v>
       </x:c>
@@ -1620,16 +2220,14 @@
         <x:v>Form không được gửi; thông báo bắt buộc rõ ràng xuất hiện phía trên nút “Cập nhật” và gắn với trường Họ Tên. FR-04, FR-22.</x:v>
       </x:c>
       <x:c r="G21" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H21" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I21" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-006 — Không có thông báo validation inline phía trên nút và không liên kết lỗi với trường.</x:v>
+      </x:c>
+      <x:c r="I21" s="27" t="str"/>
+    </x:row>
+    <x:row r="22" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A22" s="27" t="str">
         <x:v>GUI-021</x:v>
       </x:c>
@@ -1649,16 +2247,14 @@
         <x:v>Giá trị được chấp nhận và yêu cầu cập nhật được phép gửi. FR-04.</x:v>
       </x:c>
       <x:c r="G22" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H22" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I22" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-007 — Số hợp lệ 0987654321 bị từ chối; DB giữ giá trị cũ.</x:v>
+      </x:c>
+      <x:c r="I22" s="27" t="str"/>
+    </x:row>
+    <x:row r="23" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A23" s="27" t="str">
         <x:v>GUI-022</x:v>
       </x:c>
@@ -1678,16 +2274,14 @@
         <x:v>Giá trị được chấp nhận và yêu cầu cập nhật được phép gửi. FR-04.</x:v>
       </x:c>
       <x:c r="G23" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H23" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I23" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-007 — Số hợp lệ 09876543210 bị từ chối; DB giữ giá trị cũ.</x:v>
+      </x:c>
+      <x:c r="I23" s="27" t="str"/>
+    </x:row>
+    <x:row r="24" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A24" s="27" t="str">
         <x:v>GUI-023</x:v>
       </x:c>
@@ -1707,16 +2301,14 @@
         <x:v>Form không gửi dữ liệu; thông báo nêu rõ số điện thoại phải bắt đầu bằng 0. FR-04.</x:v>
       </x:c>
       <x:c r="G24" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H24" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I24" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-007 — Số 912345678 không bắt đầu bằng 0 vẫn được chấp nhận và lưu.</x:v>
+      </x:c>
+      <x:c r="I24" s="27" t="str"/>
+    </x:row>
+    <x:row r="25" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A25" s="27" t="str">
         <x:v>GUI-024</x:v>
       </x:c>
@@ -1736,16 +2328,14 @@
         <x:v>Form không gửi dữ liệu; thông báo nêu rõ độ dài hợp lệ là 10–11 chữ số. FR-04.</x:v>
       </x:c>
       <x:c r="G25" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H25" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I25" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-007 — Giá trị 9 chữ số 912345678 được chấp nhận trái FR-04.</x:v>
+      </x:c>
+      <x:c r="I25" s="27" t="str"/>
+    </x:row>
+    <x:row r="26" ht="51" hidden="0" customHeight="1">
       <x:c r="A26" s="27" t="str">
         <x:v>GUI-025</x:v>
       </x:c>
@@ -1765,16 +2355,16 @@
         <x:v>Form không gửi dữ liệu; thông báo cho biết trường chỉ chấp nhận chữ số theo định dạng của FR-04.</x:v>
       </x:c>
       <x:c r="G26" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H26" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Dữ liệu chữ abc bị từ chối; giá trị các trường khác không bị xóa.</x:v>
       </x:c>
       <x:c r="I26" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="48" hidden="0" customHeight="1">
+    <x:row r="27" ht="51" hidden="0" customHeight="1">
       <x:c r="A27" s="27" t="str">
         <x:v>GUI-026</x:v>
       </x:c>
@@ -1794,16 +2384,16 @@
         <x:v>Heuristic: Các giá trị hợp lệ ở Họ Tên và Địa chỉ vẫn được giữ nguyên để người dùng chỉ sửa trường lỗi.</x:v>
       </x:c>
       <x:c r="G27" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H27" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Sau lỗi validation, Họ Tên và Địa chỉ đã nhập vẫn được giữ nguyên.</x:v>
       </x:c>
       <x:c r="I27" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="48" hidden="0" customHeight="1">
+    <x:row r="28" ht="78" hidden="0" customHeight="1">
       <x:c r="A28" s="27" t="str">
         <x:v>GUI-027</x:v>
       </x:c>
@@ -1823,16 +2413,16 @@
         <x:v>Heuristic: Form có thể hoàn tất bằng bàn phím; Enter không tạo submit ngoài ý muốn khi đang nhập nhiều dòng trong Địa chỉ.</x:v>
       </x:c>
       <x:c r="G28" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H28" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Enter tại Họ Tên và Số điện thoại submit form; Enter trong Địa chỉ chỉ xuống dòng; sau khi Tab tới nút Cập nhật, Enter submit form bình thường.</x:v>
       </x:c>
       <x:c r="I28" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="48" hidden="0" customHeight="1">
+    <x:row r="29" ht="51" hidden="0" customHeight="1">
       <x:c r="A29" s="27" t="str">
         <x:v>GUI-028</x:v>
       </x:c>
@@ -1852,16 +2442,16 @@
         <x:v>Focus đi theo thứ tự hiển thị hợp lý; trường Email không chỉnh sửa không gây bẫy bàn phím và nút Cập nhật có thể kích hoạt bằng bàn phím. FR-21.</x:v>
       </x:c>
       <x:c r="G29" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H29" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Tab focus đúng thứ tự; khi focus ở nút Cập nhật, người dùng có thể nhấn Enter để submit.</x:v>
       </x:c>
       <x:c r="I29" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="48" hidden="0" customHeight="1">
+    <x:row r="30" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A30" s="27" t="str">
         <x:v>GUI-029</x:v>
       </x:c>
@@ -1881,16 +2471,14 @@
         <x:v>Có phản hồi thành công rõ ràng; dữ liệu vừa cập nhật hiển thị nhất quán trên Profile page. FR-04; hình thức phản hồi cụ thể là Heuristic.</x:v>
       </x:c>
       <x:c r="G30" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H30" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I30" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-007 — Không thể cập nhật với số 10–11 chữ số bắt đầu bằng 0 hợp lệ.</x:v>
+      </x:c>
+      <x:c r="I30" s="27" t="str"/>
+    </x:row>
+    <x:row r="31" ht="340.5" hidden="0" customHeight="1">
       <x:c r="A31" s="27" t="str">
         <x:v>GUI-030</x:v>
       </x:c>
@@ -1910,16 +2498,14 @@
         <x:v>Thông báo lỗi dễ hiểu xuất hiện phía trên nút “Cập nhật”; dữ liệu người dùng vừa nhập không bị xóa. FR-22; việc giữ dữ liệu là Heuristic.</x:v>
       </x:c>
       <x:c r="G31" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H31" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I31" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-018 — Lỗi PUT chỉ hiển thị bằng JavaScript alert; không có thông báo inline/aria-live, dữ liệu nhập vẫn được giữ.</x:v>
+      </x:c>
+      <x:c r="I31" s="27" t="str"/>
+    </x:row>
+    <x:row r="32" ht="51" hidden="0" customHeight="1">
       <x:c r="A32" s="56" t="str">
         <x:v>GUI-031</x:v>
       </x:c>
@@ -1939,16 +2525,16 @@
         <x:v>Mỗi đơn hiển thị Mã đơn, Ngày đặt, Tổng tiền và Trạng thái hiện tại; nhãn cột rõ ràng. FR-11.</x:v>
       </x:c>
       <x:c r="G32" s="58" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H32" s="56" t="str">
-        <x:v>—</x:v>
+        <x:v>Bảng hiển thị Mã ĐH, Ngày đặt, Tổng tiền, Trạng thái và Thao tác.</x:v>
       </x:c>
       <x:c r="I32" s="56" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="48" hidden="0" customHeight="1">
+    <x:row r="33" ht="37.5" hidden="0" customHeight="1">
       <x:c r="A33" s="27" t="str">
         <x:v>GUI-032</x:v>
       </x:c>
@@ -1968,16 +2554,16 @@
         <x:v>Mọi tổng tiền dùng ký hiệu ₫ và có phân cách hàng nghìn nhất quán. FR-11, FR-21.</x:v>
       </x:c>
       <x:c r="G33" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H33" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Tất cả tổng tiền có phân cách hàng nghìn và ký hiệu ₫.</x:v>
       </x:c>
       <x:c r="I33" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="48" hidden="0" customHeight="1">
+    <x:row r="34" ht="51" hidden="0" customHeight="1">
       <x:c r="A34" s="27" t="str">
         <x:v>GUI-033</x:v>
       </x:c>
@@ -1997,16 +2583,16 @@
         <x:v>Khu vực “Lịch sử đơn hàng” được định vị rõ trong cùng trang hoặc qua điều hướng rõ ràng; người dùng không gặp ngõ cụt. FR-11; cách tổ chức cụ thể là Heuristic.</x:v>
       </x:c>
       <x:c r="G34" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H34" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Khu vực Lịch sử đơn hàng được định vị rõ trong cùng Profile page.</x:v>
       </x:c>
       <x:c r="I34" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="48" hidden="0" customHeight="1">
+    <x:row r="35" ht="51" hidden="0" customHeight="1">
       <x:c r="A35" s="27" t="str">
         <x:v>GUI-034</x:v>
       </x:c>
@@ -2026,16 +2612,16 @@
         <x:v>Heuristic: Điều hướng trở lại đúng route; không nhân đôi đơn hàng và không hiển thị dữ liệu của phiên khác.</x:v>
       </x:c>
       <x:c r="G35" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H35" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Back về /, Forward trở lại /profile và vẫn có đúng 5 dòng đơn.</x:v>
       </x:c>
       <x:c r="I35" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="48" hidden="0" customHeight="1">
+    <x:row r="36" ht="165" hidden="0" customHeight="1">
       <x:c r="A36" s="27" t="str">
         <x:v>GUI-035</x:v>
       </x:c>
@@ -2055,16 +2641,14 @@
         <x:v>Nút có nhãn chính xác “Đăng xuất”; sau thao tác, dữ liệu đơn hàng không còn truy cập được bằng điều hướng thông thường. FR-23, SEC-02.</x:v>
       </x:c>
       <x:c r="G36" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H36" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I36" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-008 — Nút đăng xuất trên navbar ghi “Thoát” thay vì “Đăng xuất”.</x:v>
+      </x:c>
+      <x:c r="I36" s="27" t="str"/>
+    </x:row>
+    <x:row r="37" ht="164.25" hidden="0" customHeight="1">
       <x:c r="A37" s="27" t="str">
         <x:v>GUI-036</x:v>
       </x:c>
@@ -2084,16 +2668,14 @@
         <x:v>Empty state có message thân thiện và icon/hình minh họa, không chỉ là vùng trắng. FR-24.</x:v>
       </x:c>
       <x:c r="G37" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H37" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I37" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-009 — Empty state chỉ có message, không có img hoặc svg.</x:v>
+      </x:c>
+      <x:c r="I37" s="27" t="str"/>
+    </x:row>
+    <x:row r="38" ht="51" hidden="0" customHeight="1">
       <x:c r="A38" s="27" t="str">
         <x:v>GUI-037</x:v>
       </x:c>
@@ -2113,16 +2695,16 @@
         <x:v>Các trạng thái lần lượt được dịch rõ sang tiếng Việt, phân biệt màu và có nhãn văn bản để không phụ thuộc riêng vào màu. FR-11.</x:v>
       </x:c>
       <x:c r="G38" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H38" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Cả 5 trạng thái hiển thị nhãn tiếng Việt, màu riêng và văn bản trạng thái.</x:v>
       </x:c>
       <x:c r="I38" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="48" hidden="0" customHeight="1">
+    <x:row r="39" ht="165" hidden="0" customHeight="1">
       <x:c r="A39" s="27" t="str">
         <x:v>GUI-038</x:v>
       </x:c>
@@ -2142,16 +2724,14 @@
         <x:v>Heuristic: Có xác nhận trước hành động hủy; khi xác nhận và server thành công, dòng đơn cập nhật thành “Đã hủy” mà không nhân đôi dữ liệu. Việc cho phép hủy tuân FR-10.</x:v>
       </x:c>
       <x:c r="G39" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H39" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I39" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-010 — Không có confirm; alert xuất hiện sau khi đơn đã chuyển sang Đã hủy.</x:v>
+      </x:c>
+      <x:c r="I39" s="27" t="str"/>
+    </x:row>
+    <x:row r="40" ht="165" hidden="0" customHeight="1">
       <x:c r="A40" s="27" t="str">
         <x:v>GUI-039</x:v>
       </x:c>
@@ -2171,16 +2751,14 @@
         <x:v>Không hiển thị hành động tự hủy cho các trạng thái này; trạng thái kết thúc không cung cấp chuyển đổi tiếp theo. FR-10.</x:v>
       </x:c>
       <x:c r="G40" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H40" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I40" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-011 — Đơn shipping vẫn có nút Hủy đơn và hủy thành công.</x:v>
+      </x:c>
+      <x:c r="I40" s="27" t="str"/>
+    </x:row>
+    <x:row r="41" ht="51" hidden="0" customHeight="1">
       <x:c r="A41" s="56" t="str">
         <x:v>GUI-040</x:v>
       </x:c>
@@ -2200,16 +2778,16 @@
         <x:v>Màn hình dùng tiếng Việt nhất quán và có tiêu đề “Quản lý Đơn hàng” trong cấu trúc heading hợp lý. FR-21.</x:v>
       </x:c>
       <x:c r="G41" s="58" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H41" s="56" t="str">
-        <x:v>—</x:v>
+        <x:v>Mục đơn hàng có tiêu đề “Quản lý Đơn hàng” và nội dung nghiệp vụ dùng tiếng Việt.</x:v>
       </x:c>
       <x:c r="I41" s="56" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="48" hidden="0" customHeight="1">
+    <x:row r="42" ht="51" hidden="0" customHeight="1">
       <x:c r="A42" s="27" t="str">
         <x:v>GUI-041</x:v>
       </x:c>
@@ -2229,16 +2807,16 @@
         <x:v>Các cột ID, Người đặt, Tổng tiền, Địa chỉ, Trạng thái và Hành động căn chỉnh rõ; nội dung không chồng lấn. FR-18.</x:v>
       </x:c>
       <x:c r="G42" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H42" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Bảng desktop hiển thị đủ 6 cột, không chồng lấn ở viewport mặc định.</x:v>
       </x:c>
       <x:c r="I42" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="48" hidden="0" customHeight="1">
+    <x:row r="43" ht="180.75" hidden="0" customHeight="1">
       <x:c r="A43" s="27" t="str">
         <x:v>GUI-042</x:v>
       </x:c>
@@ -2258,16 +2836,14 @@
         <x:v>Địa chỉ được hiển thị như văn bản thuần, không render HTML và không thực thi script. FR-18, SEC-04.</x:v>
       </x:c>
       <x:c r="G43" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H43" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I43" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-012 — Địa chỉ chứa thẻ b được render thành HTML trong ô bảng.</x:v>
+      </x:c>
+      <x:c r="I43" s="27" t="str"/>
+    </x:row>
+    <x:row r="44" ht="51" hidden="0" customHeight="1">
       <x:c r="A44" s="27" t="str">
         <x:v>GUI-043</x:v>
       </x:c>
@@ -2287,16 +2863,16 @@
         <x:v>Mục đơn hàng được highlight và nội dung “Quản lý Đơn hàng” xuất hiện; không mở tab trình duyệt ngoài ý muốn. FR-23.</x:v>
       </x:c>
       <x:c r="G44" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H44" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Mục Đơn hàng được highlight và nội dung xuất hiện trong cùng tab.</x:v>
       </x:c>
       <x:c r="I44" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="48" hidden="0" customHeight="1">
+    <x:row r="45" ht="51" hidden="0" customHeight="1">
       <x:c r="A45" s="27" t="str">
         <x:v>GUI-044</x:v>
       </x:c>
@@ -2316,16 +2892,16 @@
         <x:v>Quyền truy cập bị từ chối và không hiển thị danh sách đơn hàng toàn hệ thống. FR-12, SEC-03.</x:v>
       </x:c>
       <x:c r="G45" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H45" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>BUG-013 — Token role=user gọi /api/admin/orders nhận 200 và 5 đơn.</x:v>
       </x:c>
       <x:c r="I45" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="48" hidden="0" customHeight="1">
+        <x:v>Bằng chứng API/authorization được ghi trong BUG-013.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="51" hidden="0" customHeight="1">
       <x:c r="A46" s="27" t="str">
         <x:v>GUI-045</x:v>
       </x:c>
@@ -2345,16 +2921,16 @@
         <x:v>Heuristic: Sidebar giữ điều hướng nhất quán; bảng đơn hàng được hiển thị lại đúng và không tạo hàng trùng.</x:v>
       </x:c>
       <x:c r="G46" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H46" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Chuyển Dashboard → Đơn hàng hiển thị lại đúng 5 dòng, không nhân đôi.</x:v>
       </x:c>
       <x:c r="I46" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="48" hidden="0" customHeight="1">
+    <x:row r="47" ht="51" hidden="0" customHeight="1">
       <x:c r="A47" s="27" t="str">
         <x:v>GUI-046</x:v>
       </x:c>
@@ -2374,16 +2950,16 @@
         <x:v>Sau phản hồi thành công, nhãn trạng thái và tập nút hành động của đúng dòng được cập nhật theo State Machine. FR-10, FR-18.</x:v>
       </x:c>
       <x:c r="G47" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H47" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Chuyển pending → confirmed cập nhật đúng nhãn và nút hành động của dòng.</x:v>
       </x:c>
       <x:c r="I47" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="48" hidden="0" customHeight="1">
+    <x:row r="48" ht="180.75" hidden="0" customHeight="1">
       <x:c r="A48" s="27" t="str">
         <x:v>GUI-047</x:v>
       </x:c>
@@ -2403,16 +2979,14 @@
         <x:v>Không có hành động chuyển sang trạng thái khác vì delivered và canceled là trạng thái kết thúc. FR-10, FR-18.</x:v>
       </x:c>
       <x:c r="G48" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H48" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I48" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-014 — Đơn canceled có nút Đánh dấu Đã giao và chuyển sang delivered thành công.</x:v>
+      </x:c>
+      <x:c r="I48" s="27" t="str"/>
+    </x:row>
+    <x:row r="49" ht="78" hidden="0" customHeight="1">
       <x:c r="A49" s="27" t="str">
         <x:v>GUI-048</x:v>
       </x:c>
@@ -2432,16 +3006,16 @@
         <x:v>Màn hình hiển thị lỗi phù hợp, giữ nguyên trạng thái hiện tại và không tạo ấn tượng rằng cập nhật đã thành công. FR-10, FR-18.</x:v>
       </x:c>
       <x:c r="G49" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H49" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Tạo race có kiểm soát: UI còn hiển thị pending nhưng DB đã delivered; thao tác Xác nhận bị API từ chối và UI không hiển thị thành công giả.</x:v>
       </x:c>
       <x:c r="I49" s="27" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="48" hidden="0" customHeight="1">
+    <x:row r="50" ht="180.75" hidden="0" customHeight="1">
       <x:c r="A50" s="56" t="str">
         <x:v>GUI-049</x:v>
       </x:c>
@@ -2461,16 +3035,14 @@
         <x:v>Nút hành động tích cực dùng màu xanh dương; nút hủy/nguy hiểm dùng màu đỏ và không chỉ dựa vào màu để truyền đạt ý nghĩa. FR-21; phần không chỉ dựa vào màu là Heuristic.</x:v>
       </x:c>
       <x:c r="G50" s="58" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H50" s="56" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I50" s="56" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-015 — Nút Hủy trong Admin dùng bg-gray-400 thay vì màu đỏ.</x:v>
+      </x:c>
+      <x:c r="I50" s="56" t="str"/>
+    </x:row>
+    <x:row r="51" ht="165" hidden="0" customHeight="1">
       <x:c r="A51" s="27" t="str">
         <x:v>GUI-050</x:v>
       </x:c>
@@ -2490,16 +3062,14 @@
         <x:v>Cùng một đích hoặc hành động dùng nhãn tiếng Việt nhất quán; hành động đăng xuất luôn ghi “Đăng xuất”. FR-21, FR-23.</x:v>
       </x:c>
       <x:c r="G51" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H51" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I51" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="48" hidden="0" customHeight="1">
+        <x:v>BUG-008 — Web User dùng nhãn “Thoát”, không nhất quán với “Đăng xuất”.</x:v>
+      </x:c>
+      <x:c r="I51" s="27" t="str"/>
+    </x:row>
+    <x:row r="52" ht="51" hidden="0" customHeight="1">
       <x:c r="A52" s="27" t="str">
         <x:v>GUI-051</x:v>
       </x:c>
@@ -2519,16 +3089,16 @@
         <x:v>Heuristic: Focus được đặt tại vị trí hợp lý để thông báo nội dung mới; người dùng không phải duyệt lại toàn bộ vùng điều hướng.</x:v>
       </x:c>
       <x:c r="G52" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H52" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>BUG-016 — Sidebar Admin không focus được; sau đổi tab activeElement vẫn là BODY.</x:v>
       </x:c>
       <x:c r="I52" s="27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="48" hidden="0" customHeight="1">
+        <x:v>Bằng chứng kiểm tra focus/DOM được ghi trong BUG-016.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="51" hidden="0" customHeight="1">
       <x:c r="A53" s="27" t="str">
         <x:v>GUI-052</x:v>
       </x:c>
@@ -2548,13 +3118,13 @@
         <x:v>Heuristic: Thông báo thành công, lỗi hoặc trạng thái đơn vừa đổi được công bố theo cách có thể cảm nhận mà không cần di chuyển focus thủ công để tìm.</x:v>
       </x:c>
       <x:c r="G53" s="29" t="str">
-        <x:v>Chưa thực hiện</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H53" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>BUG-017 — Không có role=status/alert hoặc aria-live sau thay đổi trạng thái.</x:v>
       </x:c>
       <x:c r="I53" s="27" t="str">
-        <x:v>—</x:v>
+        <x:v>Bằng chứng kiểm tra ARIA/DOM được ghi trong BUG-017.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2564,229 +3134,13 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G2:G53">
-      <x:formula1>"Chưa thực hiện,Passed,Failed"</x:formula1>
+      <x:formula1>"Passed,Failed,Chưa thực hiện"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra263c85db07b40bc"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc105eff7953c4bd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53497974afb94902"/>
   </x:tableParts>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="45" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>PHẢN BIỆN THỦ CÔNG</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="3"/>
-      <x:c r="B2" s="3"/>
-      <x:c r="C2" s="3"/>
-      <x:c r="D2" s="3"/>
-      <x:c r="E2" s="3"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>Màn hình</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>Câu hỏi phản biện độc lập</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>Gợi ý quan sát</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A5" s="24" t="str">
-        <x:v>Profile page</x:v>
-      </x:c>
-      <x:c r="B5" s="24" t="str">
-        <x:v>Có thông tin cá nhân nào hiển thị sai người dùng sau khi đổi tài khoản hoặc dùng Back không?</x:v>
-      </x:c>
-      <x:c r="C5" s="24" t="str">
-        <x:v>Thử hai tài khoản trong các phiên liên tiếp; không điền sẵn kết luận.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A6" s="25" t="str">
-        <x:v>Profile page</x:v>
-      </x:c>
-      <x:c r="B6" s="25" t="str">
-        <x:v>Khi zoom, đổi kích thước hoặc dùng bàn phím, trở ngại nào chưa được checklist AI mô tả?</x:v>
-      </x:c>
-      <x:c r="C6" s="25" t="str">
-        <x:v>Ghi lại vị trí, viewport và thao tác tái hiện.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A7" s="25" t="str">
-        <x:v>Update profile form</x:v>
-      </x:c>
-      <x:c r="B7" s="25" t="str">
-        <x:v>Quy tắc bắt buộc đối với Số điện thoại và Địa chỉ có được UI giải thích nhất quán với SRS không?</x:v>
-      </x:c>
-      <x:c r="C7" s="25" t="str">
-        <x:v>Phân biệt thiếu đặc tả với lỗi triển khai.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A8" s="25" t="str">
-        <x:v>Update profile form</x:v>
-      </x:c>
-      <x:c r="B8" s="25" t="str">
-        <x:v>Có chuỗi Unicode, dấu tiếng Việt hoặc dữ liệu dài nào làm form sai bố cục hay sai dữ liệu?</x:v>
-      </x:c>
-      <x:c r="C8" s="25" t="str">
-        <x:v>Nêu chính xác dữ liệu thử và kết quả quan sát.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A9" s="25" t="str">
-        <x:v>Order history screen</x:v>
-      </x:c>
-      <x:c r="B9" s="25" t="str">
-        <x:v>Người dùng có thể hiểu mọi trạng thái và hành động mà không dựa riêng vào màu không?</x:v>
-      </x:c>
-      <x:c r="C9" s="25" t="str">
-        <x:v>Kiểm tra nhãn, tương phản và trạng thái focus.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A10" s="25" t="str">
-        <x:v>Order history screen</x:v>
-      </x:c>
-      <x:c r="B10" s="25" t="str">
-        <x:v>Sau hủy đơn, thứ tự, trạng thái và tổng tiền có cập nhật đúng mà không cần refresh thủ công không?</x:v>
-      </x:c>
-      <x:c r="C10" s="25" t="str">
-        <x:v>So sánh trước/sau và kiểm tra đúng dòng.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A11" s="25" t="str">
-        <x:v>Admin order management</x:v>
-      </x:c>
-      <x:c r="B11" s="25" t="str">
-        <x:v>UI có cho phép chuyển trạng thái trái FR-10 hoặc làm thay đổi nhầm đơn hàng không?</x:v>
-      </x:c>
-      <x:c r="C11" s="25" t="str">
-        <x:v>Thử từng trạng thái nguồn, chỉ ghi kết quả đã quan sát.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A12" s="25" t="str">
-        <x:v>Admin order management</x:v>
-      </x:c>
-      <x:c r="B12" s="25" t="str">
-        <x:v>Dữ liệu tên người đặt hoặc địa chỉ có gây tràn bảng, render HTML hay làm mất khả năng thao tác không?</x:v>
-      </x:c>
-      <x:c r="C12" s="25" t="str">
-        <x:v>Dùng dữ liệu dài và dữ liệu chứa markup an toàn trong môi trường test.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="51" t="str">
-        <x:v>MỤC DO SINH VIÊN BỔ SUNG — để trống; không xem gợi ý AI là đóng góp của sinh viên</x:v>
-      </x:c>
-      <x:c r="B14" s="51"/>
-      <x:c r="C14" s="51"/>
-      <x:c r="D14" s="51"/>
-      <x:c r="E14" s="51"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="9" t="str">
-        <x:v>ID sinh viên</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="str">
-        <x:v>Màn hình</x:v>
-      </x:c>
-      <x:c r="C16" s="9" t="str">
-        <x:v>Mục kiểm tra bổ sung</x:v>
-      </x:c>
-      <x:c r="D16" s="9" t="str">
-        <x:v>Vì sao AI bỏ sót</x:v>
-      </x:c>
-      <x:c r="E16" s="9" t="str">
-        <x:v>Kết quả/ghi chú khi thực thi</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="34" customHeight="1">
-      <x:c r="A17" s="55" t="str"/>
-      <x:c r="B17" s="55" t="str"/>
-      <x:c r="C17" s="55" t="str"/>
-      <x:c r="D17" s="55" t="str"/>
-      <x:c r="E17" s="55" t="str"/>
-    </x:row>
-    <x:row r="18" ht="34" customHeight="1">
-      <x:c r="A18" s="55" t="str"/>
-      <x:c r="B18" s="55" t="str"/>
-      <x:c r="C18" s="55" t="str"/>
-      <x:c r="D18" s="55" t="str"/>
-      <x:c r="E18" s="55" t="str"/>
-    </x:row>
-    <x:row r="19" ht="34" customHeight="1">
-      <x:c r="A19" s="55" t="str"/>
-      <x:c r="B19" s="55" t="str"/>
-      <x:c r="C19" s="55" t="str"/>
-      <x:c r="D19" s="55" t="str"/>
-      <x:c r="E19" s="55" t="str"/>
-    </x:row>
-    <x:row r="20" ht="34" customHeight="1">
-      <x:c r="A20" s="55" t="str"/>
-      <x:c r="B20" s="55" t="str"/>
-      <x:c r="C20" s="55" t="str"/>
-      <x:c r="D20" s="55" t="str"/>
-      <x:c r="E20" s="55" t="str"/>
-    </x:row>
-    <x:row r="21" ht="34" customHeight="1">
-      <x:c r="A21" s="55" t="str"/>
-      <x:c r="B21" s="55" t="str"/>
-      <x:c r="C21" s="55" t="str"/>
-      <x:c r="D21" s="55" t="str"/>
-      <x:c r="E21" s="55" t="str"/>
-    </x:row>
-    <x:row r="22" ht="34" customHeight="1">
-      <x:c r="A22" s="55" t="str"/>
-      <x:c r="B22" s="55" t="str"/>
-      <x:c r="C22" s="55" t="str"/>
-      <x:c r="D22" s="55" t="str"/>
-      <x:c r="E22" s="55" t="str"/>
-    </x:row>
-    <x:row r="23" ht="34" customHeight="1">
-      <x:c r="A23" s="55" t="str"/>
-      <x:c r="B23" s="55" t="str"/>
-      <x:c r="C23" s="55" t="str"/>
-      <x:c r="D23" s="55" t="str"/>
-      <x:c r="E23" s="55" t="str"/>
-    </x:row>
-    <x:row r="24" ht="34" customHeight="1">
-      <x:c r="A24" s="55" t="str"/>
-      <x:c r="B24" s="55" t="str"/>
-      <x:c r="C24" s="55" t="str"/>
-      <x:c r="D24" s="55" t="str"/>
-      <x:c r="E24" s="55" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:E2"/>
-    <x:mergeCell ref="A14:E14"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>